<commit_message>
Update warehouse/warehouse.xlsx via NBS Ad Tracker
</commit_message>
<xml_diff>
--- a/warehouse/warehouse.xlsx
+++ b/warehouse/warehouse.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5051,7 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6001,7 +6001,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6051,7 +6051,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6151,7 +6151,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6251,7 +6251,7 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6401,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6451,7 +6451,7 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6501,7 +6501,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6751,7 +6751,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6851,7 +6851,7 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -6951,7 +6951,7 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7001,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -7051,7 +7051,7 @@
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -7101,7 +7101,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D454"/>
+  <dimension ref="A1:D534"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17155,6 +17155,1766 @@
         </is>
       </c>
       <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Row 1 (Monday)</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>NALU COSMETICS SQ BK</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'NALU COSMETICS SQZBK' (95.0%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>Row 2 (Monday)</t>
+        </is>
+      </c>
+      <c r="B456" s="2" t="inlineStr">
+        <is>
+          <t>SUNRISE DIGEST</t>
+        </is>
+      </c>
+      <c r="C456" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Row 6 (Monday)</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>WAKE UP UGANDA</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>Row 10 (Monday)</t>
+        </is>
+      </c>
+      <c r="B458" s="2" t="inlineStr">
+        <is>
+          <t>BREAKFAST BITES</t>
+        </is>
+      </c>
+      <c r="C458" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Row 12 (Monday)</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>BRIGHTWAVE SQ BK</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>Row 13 (Monday)</t>
+        </is>
+      </c>
+      <c r="B460" s="2" t="inlineStr">
+        <is>
+          <t>AM DRIVE</t>
+        </is>
+      </c>
+      <c r="C460" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Row 15 (Monday)</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>CITY PULSE</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>Row 18 (Monday)</t>
+        </is>
+      </c>
+      <c r="B462" s="2" t="inlineStr">
+        <is>
+          <t>AMARA SKINCARE TVC</t>
+        </is>
+      </c>
+      <c r="C462" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'AMARA SKINCARE' (95.0%) - assigned Trade Marketing</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Row 21 (Monday)</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>EMERALDTEL SQ BK</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>Row 22 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B464" s="2" t="inlineStr">
+        <is>
+          <t>ZENGLOW TVC</t>
+        </is>
+      </c>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Row 24 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>SUNRISE DIGEST</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>Row 25 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B466" s="2" t="inlineStr">
+        <is>
+          <t>ROLEX EXPRESS TVC</t>
+        </is>
+      </c>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'ROLEX EXPRESS' (95.0%) - assigned Swap</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Row 29 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>ZAWADI FASHION SQ BK</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'ZAWADI FASHION SQZBK' (95.0%) - assigned Swap</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>Row 30 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B468" s="2" t="inlineStr">
+        <is>
+          <t>WAKE UP UGANDA</t>
+        </is>
+      </c>
+      <c r="C468" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Row 31 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>CRESTLINE FOODS SQ BK</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CRESTLINE FOODS SQZBK' (95.2%) - assigned Commercial</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>Row 32 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B470" s="2" t="inlineStr">
+        <is>
+          <t>RIDGEWAY FURNITURE TVC</t>
+        </is>
+      </c>
+      <c r="C470" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'RIDGEWAY FURNITURE' (95.0%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Row 33 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>BREAKFAST BITES</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>Row 36 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B472" s="2" t="inlineStr">
+        <is>
+          <t>AM DRIVE</t>
+        </is>
+      </c>
+      <c r="C472" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Row 37 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>NYATI MOTORS PROMO</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>Row 38 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B474" s="2" t="inlineStr">
+        <is>
+          <t>CITY PULSE</t>
+        </is>
+      </c>
+      <c r="C474" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Row 42 (Tuesday)</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>NALU COSMETICS SQ BK</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'NALU COSMETICS SQZBK' (95.0%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>Row 46 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B476" s="2" t="inlineStr">
+        <is>
+          <t>BRIGHTWAVE SQ BK</t>
+        </is>
+      </c>
+      <c r="C476" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>Row 47 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>SUNRISE DIGEST</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="inlineStr">
+        <is>
+          <t>Row 51 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B478" s="2" t="inlineStr">
+        <is>
+          <t>BRIGHTWAVE SQ BK</t>
+        </is>
+      </c>
+      <c r="C478" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Row 52 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>WAKE UP UGANDA</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="inlineStr">
+        <is>
+          <t>Row 53 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B480" s="2" t="inlineStr">
+        <is>
+          <t>TERALINK SQ BK</t>
+        </is>
+      </c>
+      <c r="C480" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D480" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Row 54 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>BRIGHTWAVE SQ BK</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="inlineStr">
+        <is>
+          <t>Row 55 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B482" s="2" t="inlineStr">
+        <is>
+          <t>BREAKFAST BITES</t>
+        </is>
+      </c>
+      <c r="C482" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Row 58 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>AMARA SKINCARE TVC</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'AMARA SKINCARE' (95.0%) - assigned Trade Marketing</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="inlineStr">
+        <is>
+          <t>Row 60 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B484" s="2" t="inlineStr">
+        <is>
+          <t>CEDAR GROVE REALTY SQ BK</t>
+        </is>
+      </c>
+      <c r="C484" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CEDAR GROVE REALTY SQZBK' (95.8%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D484" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Row 61 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>AM DRIVE</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="inlineStr">
+        <is>
+          <t>Row 62 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B486" s="2" t="inlineStr">
+        <is>
+          <t>TERALINK SQ BK</t>
+        </is>
+      </c>
+      <c r="C486" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D486" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Row 63 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>CRESTLINE FOODS SQ BK</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CRESTLINE FOODS SQZBK' (95.2%) - assigned Commercial</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>Row 64 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B488" s="2" t="inlineStr">
+        <is>
+          <t>TWIGA AIRTIME TVC</t>
+        </is>
+      </c>
+      <c r="C488" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'TWIGA AIRTIME' (95.0%) - assigned Commercial</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Row 65 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>CITY PULSE</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>Row 66 (Wednesday)</t>
+        </is>
+      </c>
+      <c r="B490" s="2" t="inlineStr">
+        <is>
+          <t>ZENGLOW TVC</t>
+        </is>
+      </c>
+      <c r="C490" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Row 67 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>CRESTLINE FOODS SQ BK</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CRESTLINE FOODS SQZBK' (95.2%) - assigned Commercial</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="inlineStr">
+        <is>
+          <t>Row 68 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B492" s="2" t="inlineStr">
+        <is>
+          <t>SUNRISE DIGEST</t>
+        </is>
+      </c>
+      <c r="C492" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Row 69 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>AMARA SKINCARE TVC</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'AMARA SKINCARE' (95.0%) - assigned Trade Marketing</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="inlineStr">
+        <is>
+          <t>Row 70 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B494" s="2" t="inlineStr">
+        <is>
+          <t>WAKE UP UGANDA</t>
+        </is>
+      </c>
+      <c r="C494" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Row 72 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>BREAKFAST BITES</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="inlineStr">
+        <is>
+          <t>Row 74 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B496" s="2" t="inlineStr">
+        <is>
+          <t>ZENGLOW TVC</t>
+        </is>
+      </c>
+      <c r="C496" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Row 75 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>RIDGEWAY FURNITURE TVC</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'RIDGEWAY FURNITURE' (95.0%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="inlineStr">
+        <is>
+          <t>Row 76 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B498" s="2" t="inlineStr">
+        <is>
+          <t>AMARA SKINCARE TVC</t>
+        </is>
+      </c>
+      <c r="C498" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'AMARA SKINCARE' (95.0%) - assigned Trade Marketing</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Row 78 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>CRESTLINE FOODS SQ BK</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CRESTLINE FOODS SQZBK' (95.2%) - assigned Commercial</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="inlineStr">
+        <is>
+          <t>Row 80 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B500" s="2" t="inlineStr">
+        <is>
+          <t>AM DRIVE</t>
+        </is>
+      </c>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Row 82 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>EMERALDTEL SQ BK</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="inlineStr">
+        <is>
+          <t>Row 83 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B502" s="2" t="inlineStr">
+        <is>
+          <t>CITY PULSE</t>
+        </is>
+      </c>
+      <c r="C502" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Row 84 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>CEDAR GROVE REALTY SQ BK</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CEDAR GROVE REALTY SQZBK' (95.8%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>Row 86 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B504" s="2" t="inlineStr">
+        <is>
+          <t>HIGHLAND BREW TVC</t>
+        </is>
+      </c>
+      <c r="C504" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Row 88 (Thursday)</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>PEMBA TYRES PROMO</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="inlineStr">
+        <is>
+          <t>Row 91 (Friday)</t>
+        </is>
+      </c>
+      <c r="B506" s="2" t="inlineStr">
+        <is>
+          <t>CRESTLINE FOODS SQ BK</t>
+        </is>
+      </c>
+      <c r="C506" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CRESTLINE FOODS SQZBK' (95.2%) - assigned Commercial</t>
+        </is>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Row 92 (Friday)</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>RIDGEWAY FURNITURE TVC</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'RIDGEWAY FURNITURE' (95.0%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="inlineStr">
+        <is>
+          <t>Row 93 (Friday)</t>
+        </is>
+      </c>
+      <c r="B508" s="2" t="inlineStr">
+        <is>
+          <t>RIDGEWAY FURNITURE TVC</t>
+        </is>
+      </c>
+      <c r="C508" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'RIDGEWAY FURNITURE' (95.0%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Row 94 (Friday)</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>RIDGEWAY FURNITURE TVC</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'RIDGEWAY FURNITURE' (95.0%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>Row 95 (Friday)</t>
+        </is>
+      </c>
+      <c r="B510" s="2" t="inlineStr">
+        <is>
+          <t>SUNRISE DIGEST</t>
+        </is>
+      </c>
+      <c r="C510" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Row 97 (Friday)</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>AMARA SKINCARE TVC</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'AMARA SKINCARE' (95.0%) - assigned Trade Marketing</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="inlineStr">
+        <is>
+          <t>Row 98 (Friday)</t>
+        </is>
+      </c>
+      <c r="B512" s="2" t="inlineStr">
+        <is>
+          <t>WAKE UP UGANDA</t>
+        </is>
+      </c>
+      <c r="C512" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Row 99 (Friday)</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>PEMBA TYRES PROMO</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>Row 100 (Friday)</t>
+        </is>
+      </c>
+      <c r="B514" s="2" t="inlineStr">
+        <is>
+          <t>BRIGHTWAVE SQ BK</t>
+        </is>
+      </c>
+      <c r="C514" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Row 101 (Friday)</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>BREAKFAST BITES</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>Row 102 (Friday)</t>
+        </is>
+      </c>
+      <c r="B516" s="2" t="inlineStr">
+        <is>
+          <t>ROLEX EXPRESS TVC</t>
+        </is>
+      </c>
+      <c r="C516" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'ROLEX EXPRESS' (95.0%) - assigned Swap</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Row 103 (Friday)</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>CEDAR GROVE REALTY SQ BK</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CEDAR GROVE REALTY SQZBK' (95.8%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>Row 104 (Friday)</t>
+        </is>
+      </c>
+      <c r="B518" s="2" t="inlineStr">
+        <is>
+          <t>HIGHLAND BREW TVC</t>
+        </is>
+      </c>
+      <c r="C518" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Row 105 (Friday)</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>NYATI MOTORS PROMO</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>Row 106 (Friday)</t>
+        </is>
+      </c>
+      <c r="B520" s="2" t="inlineStr">
+        <is>
+          <t>RIDGEWAY FURNITURE TVC</t>
+        </is>
+      </c>
+      <c r="C520" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'RIDGEWAY FURNITURE' (95.0%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Row 107 (Friday)</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>ROLEX EXPRESS TVC</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'ROLEX EXPRESS' (95.0%) - assigned Swap</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>Row 108 (Friday)</t>
+        </is>
+      </c>
+      <c r="B522" s="2" t="inlineStr">
+        <is>
+          <t>AM DRIVE</t>
+        </is>
+      </c>
+      <c r="C522" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Row 110 (Friday)</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>CITY PULSE</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>Row 113 (Friday)</t>
+        </is>
+      </c>
+      <c r="B524" s="2" t="inlineStr">
+        <is>
+          <t>TERALINK SQ BK</t>
+        </is>
+      </c>
+      <c r="C524" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Row 115 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>SUNRISE DIGEST</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="inlineStr">
+        <is>
+          <t>Row 117 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B526" s="2" t="inlineStr">
+        <is>
+          <t>WAKE UP UGANDA</t>
+        </is>
+      </c>
+      <c r="C526" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Row 118 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>EMERALDTEL SQ BK</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>Row 120 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="inlineStr">
+        <is>
+          <t>HIGHLAND BREW TVC</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Row 121 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>CEDAR GROVE REALTY SQ BK</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CEDAR GROVE REALTY SQZBK' (95.8%) - assigned Internal</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>Row 122 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B530" s="2" t="inlineStr">
+        <is>
+          <t>CRESTLINE FOODS SQ BK</t>
+        </is>
+      </c>
+      <c r="C530" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CRESTLINE FOODS SQZBK' (95.2%) - assigned Commercial</t>
+        </is>
+      </c>
+      <c r="D530" s="2" t="inlineStr">
+        <is>
+          <t>Confirm match is correct in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Row 126 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>NYATI MOTORS PROMO</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>Row 129 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B532" s="2" t="inlineStr">
+        <is>
+          <t>EMERALDTEL SQ BK</t>
+        </is>
+      </c>
+      <c r="C532" s="2" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D532" s="2" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Row 130 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>BREAKFAST BITES</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>No category match found</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Assign category in Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>Row 131 (Saturday)</t>
+        </is>
+      </c>
+      <c r="B534" s="2" t="inlineStr">
+        <is>
+          <t>CRESTLINE FOODS SQ BK</t>
+        </is>
+      </c>
+      <c r="C534" s="2" t="inlineStr">
+        <is>
+          <t>Fuzzy matched to 'CRESTLINE FOODS SQZBK' (95.2%) - assigned Commercial</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
         <is>
           <t>Confirm match is correct in Mapping Manager</t>
         </is>
@@ -18046,7 +19806,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>453</v>
+        <v>533</v>
       </c>
     </row>
     <row r="8">
@@ -18067,7 +19827,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30.07.2026 16:03</t>
+          <t>30.07.2026 16:04</t>
         </is>
       </c>
     </row>

</xml_diff>